<commit_message>
xml serializing working, adding unique sign list func
</commit_message>
<xml_diff>
--- a/010-npm_node/02-results/2106G14RS Broadstone Trinity REV 3.xlsx
+++ b/010-npm_node/02-results/2106G14RS Broadstone Trinity REV 3.xlsx
@@ -464,7 +464,7 @@
         <v>CONTACT</v>
       </c>
       <c r="I2" t="str">
-        <v>CONTRACT_NUMBER</v>
+        <v>CONTRACT</v>
       </c>
       <c r="J2" t="str">
         <v>REVISIONS</v>
@@ -476,7 +476,7 @@
         <v>CONTRACT_FILE</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" xml:space="preserve">
       <c r="A3" t="str">
         <v>#1: ENTRY SIGNAGE</v>
       </c>
@@ -504,8 +504,11 @@
       <c r="I3" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J3" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J3" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K3" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -514,7 +517,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" xml:space="preserve">
       <c r="A4" t="str">
         <v>#1: ENTRY SIGNAGE</v>
       </c>
@@ -542,8 +545,11 @@
       <c r="I4" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J4" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J4" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K4" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -552,7 +558,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -580,8 +586,11 @@
       <c r="I5" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J5" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J5" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K5" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -590,7 +599,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" xml:space="preserve">
       <c r="A6" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -618,8 +627,11 @@
       <c r="I6" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J6" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J6" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K6" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -628,7 +640,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" xml:space="preserve">
       <c r="A7" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -656,8 +668,11 @@
       <c r="I7" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J7" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J7" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K7" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -666,7 +681,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" xml:space="preserve">
       <c r="A8" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -694,8 +709,11 @@
       <c r="I8" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J8" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J8" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K8" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -704,7 +722,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" xml:space="preserve">
       <c r="A9" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -732,8 +750,11 @@
       <c r="I9" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J9" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J9" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K9" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -742,7 +763,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" xml:space="preserve">
       <c r="A10" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -770,8 +791,11 @@
       <c r="I10" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J10" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J10" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K10" t="str">
         <v>BROADSTONE TRINITY</v>
@@ -780,7 +804,7 @@
         <v>2106G14RS Broadstone Trinity REV 3.xlsx</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" xml:space="preserve">
       <c r="A11" t="str">
         <v>#2: LEASING CENTER- EXTERIOR / INTERIOR SIGNAGE</v>
       </c>
@@ -808,8 +832,11 @@
       <c r="I11" t="str">
         <v>2106G14RS</v>
       </c>
-      <c r="J11" t="str">
-        <v>07.02.21 08.23.2021 REVISION 1 10.15.2021 REVISION 2 11.12.2021 REVISION 3</v>
+      <c r="J11" t="str" xml:space="preserve">
+        <v xml:space="preserve">07.02.21 08.23.2021 REVISION 1
+ 10.15.2021 REVISION 2
+ 11.12.2021 REVISION 3
+</v>
       </c>
       <c r="K11" t="str">
         <v>BROADSTONE TRINITY</v>

</xml_diff>